<commit_message>
se elimina penalizacion de viaje a estacion de carga y se agrega minimo de 2 intervalos cargando
</commit_message>
<xml_diff>
--- a/data/Escenarios_DCH_costos_nuevos/Costo_fijo/Carga_on_board_fixed_3estaciones_1000kW/elmo_data.xlsx
+++ b/data/Escenarios_DCH_costos_nuevos/Costo_fijo/Carga_on_board_fixed_3estaciones_1000kW/elmo_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\Escenarios_DCH_costos_nuevos\Costo_fijo\Carga_on_board_fixed_3estaciones_1000kW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A9FA33A-F1C4-4D68-8E4F-99865D5FB2F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{291D18D3-25BA-4E3D-A3B3-91B01C3C0B8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LHD" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1080" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1076" uniqueCount="390">
   <si>
     <t>id</t>
   </si>
@@ -1158,16 +1158,7 @@
     <t>station_name</t>
   </si>
   <si>
-    <t>distance_to_dn</t>
-  </si>
-  <si>
-    <t>man_time</t>
-  </si>
-  <si>
     <t>USD</t>
-  </si>
-  <si>
-    <t>h</t>
   </si>
   <si>
     <t>station_1</t>
@@ -2317,7 +2308,7 @@
         <v>40</v>
       </c>
       <c r="C3" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="D3" s="27" t="s">
         <v>67</v>
@@ -2406,7 +2397,7 @@
         <v>63</v>
       </c>
       <c r="C4" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="D4" s="27" t="s">
         <v>67</v>
@@ -2495,7 +2486,7 @@
         <v>64</v>
       </c>
       <c r="C5" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="D5" s="27" t="s">
         <v>67</v>
@@ -2584,7 +2575,7 @@
         <v>65</v>
       </c>
       <c r="C6" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="D6" s="27" t="s">
         <v>67</v>
@@ -2673,7 +2664,7 @@
         <v>352</v>
       </c>
       <c r="C7" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="D7" s="27" t="s">
         <v>67</v>
@@ -2762,7 +2753,7 @@
         <v>353</v>
       </c>
       <c r="C8" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="D8" s="27" t="s">
         <v>67</v>
@@ -2851,7 +2842,7 @@
         <v>354</v>
       </c>
       <c r="C9" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="D9" s="27" t="s">
         <v>67</v>
@@ -2940,7 +2931,7 @@
         <v>355</v>
       </c>
       <c r="C10" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="D10" s="27" t="s">
         <v>67</v>
@@ -3029,7 +3020,7 @@
         <v>356</v>
       </c>
       <c r="C11" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="D11" s="27" t="s">
         <v>67</v>
@@ -3119,7 +3110,7 @@
         <v>357</v>
       </c>
       <c r="C12" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="D12" s="27" t="s">
         <v>67</v>
@@ -3209,7 +3200,7 @@
         <v>358</v>
       </c>
       <c r="C13" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="D13" s="27" t="s">
         <v>67</v>
@@ -3299,7 +3290,7 @@
         <v>359</v>
       </c>
       <c r="C14" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="D14" s="27" t="s">
         <v>67</v>
@@ -3392,7 +3383,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC93900-5A86-4519-AB89-460E8AC441EE}">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
@@ -3401,10 +3392,9 @@
     <col min="5" max="5" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.42578125" customWidth="1"/>
     <col min="7" max="7" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3412,31 +3402,25 @@
         <v>372</v>
       </c>
       <c r="C1" t="s">
+        <v>385</v>
+      </c>
+      <c r="D1" t="s">
+        <v>386</v>
+      </c>
+      <c r="E1" t="s">
+        <v>387</v>
+      </c>
+      <c r="F1" t="s">
         <v>388</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>389</v>
       </c>
-      <c r="E1" t="s">
-        <v>390</v>
-      </c>
-      <c r="F1" t="s">
-        <v>391</v>
-      </c>
-      <c r="G1" t="s">
-        <v>392</v>
-      </c>
       <c r="H1" t="s">
-        <v>373</v>
-      </c>
-      <c r="I1" t="s">
-        <v>374</v>
-      </c>
-      <c r="J1" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -3444,13 +3428,13 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="D2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="E2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="F2" t="s">
         <v>51</v>
@@ -3459,21 +3443,15 @@
         <v>51</v>
       </c>
       <c r="H2" t="s">
-        <v>10</v>
-      </c>
-      <c r="I2" t="s">
-        <v>376</v>
-      </c>
-      <c r="J2" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="C3">
         <v>35722</v>
@@ -3491,21 +3469,15 @@
         <v>1</v>
       </c>
       <c r="H3">
-        <v>168</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3">
         <v>1500</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="C4">
         <v>35722</v>
@@ -3523,21 +3495,15 @@
         <v>1</v>
       </c>
       <c r="H4">
-        <v>168</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
         <v>1500</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="C5">
         <v>35722</v>
@@ -3555,12 +3521,6 @@
         <v>1</v>
       </c>
       <c r="H5">
-        <v>253</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
         <v>1500</v>
       </c>
     </row>
@@ -3580,19 +3540,19 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>375</v>
+      </c>
+      <c r="C1" t="s">
+        <v>376</v>
+      </c>
+      <c r="D1" t="s">
+        <v>377</v>
+      </c>
+      <c r="E1" t="s">
         <v>378</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>379</v>
-      </c>
-      <c r="D1" t="s">
-        <v>380</v>
-      </c>
-      <c r="E1" t="s">
-        <v>381</v>
-      </c>
-      <c r="F1" t="s">
-        <v>382</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -3603,7 +3563,7 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="D2" t="s">
         <v>34</v>
@@ -3620,7 +3580,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="C3">
         <v>131400</v>

</xml_diff>